<commit_message>
chore: update fixed order export template
</commit_message>
<xml_diff>
--- a/src/assets/order-templates/ROMIKU_订单_模板.xlsx
+++ b/src/assets/order-templates/ROMIKU_订单_模板.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="32260" windowHeight="15260"/>
+    <workbookView windowHeight="15480"/>
   </bookViews>
   <sheets>
     <sheet name="ROMIKU PI" sheetId="1" r:id="rId1"/>
@@ -32,14 +32,25 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
   <si>
-    <t xml:space="preserve">                          ORDER</t>
+    <r>
+      <t xml:space="preserve">                          </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="48"/>
+        <rFont val="Songti SC Regular"/>
+        <charset val="134"/>
+      </rPr>
+      <t>ORDER</t>
+    </r>
   </si>
   <si>
     <t>ORDER.NO:
 DATE:</t>
   </si>
   <si>
-    <t>PI260923001
+    <t>OD260923001
 2026.9.22</t>
   </si>
   <si>
@@ -60,7 +71,8 @@
 地址</t>
   </si>
   <si>
-    <t>72790, 3rd Street, Unit 4, 2nd Floor, Gate 153,Global Digital Trade Center Yiwu,China</t>
+    <t>72790, 3rd Street, Unit 4, 2nd Floor, Gate 153,Global Digital Trade Center Yiwu,China
+义乌市国际商贸城六区152号门2楼4单元3街72790 </t>
   </si>
   <si>
     <t>TEL/WHATSAPP
@@ -222,7 +234,7 @@
     <numFmt numFmtId="176" formatCode="\$#,##0.00;\-\$#,##0.00"/>
     <numFmt numFmtId="177" formatCode="&quot;USD&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="36">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -241,7 +253,7 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="16"/>
       <name val="Songti SC Regular"/>
       <charset val="134"/>
     </font>
@@ -253,18 +265,24 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="20"/>
       <name val="Songti SC Regular"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="22"/>
+      <sz val="28"/>
       <name val="Songti SC Regular"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="16"/>
+      <b/>
+      <sz val="24"/>
+      <name val="Songti SC Regular"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="18"/>
       <name val="Songti SC Regular"/>
       <charset val="134"/>
     </font>
@@ -453,6 +471,12 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="48"/>
+      <name val="Songti SC Regular"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="35">
@@ -913,153 +937,153 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyFont="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
@@ -1081,31 +1105,31 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="5" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1141,34 +1165,34 @@
     <xf numFmtId="176" fontId="6" fillId="0" borderId="10" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="7" fontId="5" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="7" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="11" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="11" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1177,54 +1201,57 @@
     <xf numFmtId="176" fontId="5" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="49" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="12" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="12" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="49" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1507,16 +1534,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>760095</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>224790</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>280035</xdr:rowOff>
+      <xdr:rowOff>193040</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1090295</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1007110</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>974725</xdr:rowOff>
+      <xdr:rowOff>1099185</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1534,8 +1561,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3321050" y="280035"/>
-          <a:ext cx="2562860" cy="694690"/>
+          <a:off x="224790" y="193040"/>
+          <a:ext cx="3343275" cy="906145"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1787,7 +1814,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="9"/>
-      <c r="C5" s="58" t="s">
+      <c r="C5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="11"/>
@@ -1836,7 +1863,7 @@
       <c r="I7" s="11"/>
       <c r="J7" s="12"/>
     </row>
-    <row r="8" ht="47" customHeight="1" spans="1:10">
+    <row r="8" ht="60" customHeight="1" spans="1:10">
       <c r="A8" s="15" t="s">
         <v>15</v>
       </c>
@@ -1942,7 +1969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="35" customHeight="1" spans="1:10">
+    <row r="13" ht="45" customHeight="1" spans="1:10">
       <c r="A13" s="29" t="s">
         <v>25</v>
       </c>
@@ -1964,7 +1991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="35" customHeight="1" spans="1:10">
+    <row r="14" ht="45" customHeight="1" spans="1:10">
       <c r="A14" s="34" t="s">
         <v>27</v>
       </c>
@@ -1980,7 +2007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="35" customHeight="1" spans="1:10">
+    <row r="15" ht="45" customHeight="1" spans="1:10">
       <c r="A15" s="36" t="s">
         <v>28</v>
       </c>
@@ -1997,7 +2024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="35" customHeight="1" spans="1:10">
+    <row r="16" ht="45" customHeight="1" spans="1:10">
       <c r="A16" s="29" t="s">
         <v>29</v>
       </c>
@@ -2014,7 +2041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" ht="35" customHeight="1" spans="1:10">
+    <row r="17" ht="45" customHeight="1" spans="1:10">
       <c r="A17" s="29" t="s">
         <v>30</v>
       </c>
@@ -2031,7 +2058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="23.2" spans="1:10">
+    <row r="18" ht="30" customHeight="1" spans="1:10">
       <c r="A18" s="39" t="s">
         <v>31</v>
       </c>
@@ -2045,229 +2072,229 @@
       <c r="I18" s="40"/>
       <c r="J18" s="40"/>
     </row>
-    <row r="19" s="1" customFormat="1" ht="70" customHeight="1" spans="1:10">
+    <row r="19" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
       <c r="A19" s="41">
         <v>1</v>
       </c>
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="42"/>
-      <c r="D19" s="43" t="s">
+      <c r="C19" s="43"/>
+      <c r="D19" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="E19" s="44"/>
-      <c r="F19" s="44"/>
-      <c r="G19" s="44"/>
-      <c r="H19" s="44"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="46"/>
-    </row>
-    <row r="20" s="1" customFormat="1" ht="70" customHeight="1" spans="1:10">
+      <c r="E19" s="45"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="45"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="47"/>
+    </row>
+    <row r="20" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
       <c r="A20" s="41">
         <v>2</v>
       </c>
-      <c r="B20" s="47" t="s">
+      <c r="B20" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="48"/>
-      <c r="D20" s="43" t="s">
+      <c r="C20" s="49"/>
+      <c r="D20" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="E20" s="44"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="45"/>
-      <c r="J20" s="46"/>
-    </row>
-    <row r="21" s="1" customFormat="1" ht="70" customHeight="1" spans="1:10">
+      <c r="E20" s="45"/>
+      <c r="F20" s="45"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="45"/>
+      <c r="I20" s="46"/>
+      <c r="J20" s="47"/>
+    </row>
+    <row r="21" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
       <c r="A21" s="41">
         <v>3</v>
       </c>
-      <c r="B21" s="47" t="s">
+      <c r="B21" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="43" t="s">
+      <c r="C21" s="49"/>
+      <c r="D21" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="E21" s="44"/>
-      <c r="F21" s="44"/>
-      <c r="G21" s="44"/>
-      <c r="H21" s="44"/>
-      <c r="I21" s="44"/>
-      <c r="J21" s="46"/>
-    </row>
-    <row r="22" s="1" customFormat="1" ht="70" customHeight="1" spans="1:10">
+      <c r="E21" s="45"/>
+      <c r="F21" s="45"/>
+      <c r="G21" s="45"/>
+      <c r="H21" s="45"/>
+      <c r="I21" s="45"/>
+      <c r="J21" s="47"/>
+    </row>
+    <row r="22" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
       <c r="A22" s="41">
         <v>4</v>
       </c>
-      <c r="B22" s="47" t="s">
+      <c r="B22" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="48"/>
-      <c r="D22" s="43" t="s">
+      <c r="C22" s="49"/>
+      <c r="D22" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="44"/>
-      <c r="I22" s="44"/>
-      <c r="J22" s="46"/>
-    </row>
-    <row r="23" s="1" customFormat="1" ht="70" customHeight="1" spans="1:10">
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="45"/>
+      <c r="J22" s="47"/>
+    </row>
+    <row r="23" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
       <c r="A23" s="41">
         <v>5</v>
       </c>
-      <c r="B23" s="47" t="s">
+      <c r="B23" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="48"/>
-      <c r="D23" s="43" t="s">
+      <c r="C23" s="49"/>
+      <c r="D23" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="44"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="44"/>
-      <c r="I23" s="44"/>
-      <c r="J23" s="46"/>
-    </row>
-    <row r="24" s="1" customFormat="1" ht="70" customHeight="1" spans="1:10">
+      <c r="E23" s="45"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="45"/>
+      <c r="I23" s="45"/>
+      <c r="J23" s="47"/>
+    </row>
+    <row r="24" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
       <c r="A24" s="41">
         <v>6</v>
       </c>
-      <c r="B24" s="47" t="s">
+      <c r="B24" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="C24" s="48"/>
-      <c r="D24" s="43" t="s">
+      <c r="C24" s="49"/>
+      <c r="D24" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="E24" s="44"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="44"/>
-      <c r="I24" s="44"/>
-      <c r="J24" s="46"/>
-    </row>
-    <row r="25" s="1" customFormat="1" ht="70" customHeight="1" spans="1:10">
+      <c r="E24" s="45"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="45"/>
+      <c r="J24" s="47"/>
+    </row>
+    <row r="25" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
       <c r="A25" s="41">
         <v>7</v>
       </c>
-      <c r="B25" s="30" t="s">
+      <c r="B25" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="42"/>
-      <c r="D25" s="43" t="s">
+      <c r="C25" s="43"/>
+      <c r="D25" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="44"/>
-      <c r="F25" s="44"/>
-      <c r="G25" s="44"/>
-      <c r="H25" s="44"/>
-      <c r="I25" s="45"/>
-      <c r="J25" s="46"/>
-    </row>
-    <row r="26" s="1" customFormat="1" ht="70" customHeight="1" spans="1:10">
+      <c r="E25" s="45"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="45"/>
+      <c r="H25" s="45"/>
+      <c r="I25" s="46"/>
+      <c r="J25" s="47"/>
+    </row>
+    <row r="26" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
       <c r="A26" s="41">
         <v>8</v>
       </c>
-      <c r="B26" s="30" t="s">
+      <c r="B26" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="42"/>
-      <c r="D26" s="43" t="s">
+      <c r="C26" s="43"/>
+      <c r="D26" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="45"/>
-      <c r="J26" s="46"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="46"/>
+      <c r="J26" s="47"/>
     </row>
     <row r="27" s="1" customFormat="1" ht="24" customHeight="1" spans="1:10">
-      <c r="A27" s="49"/>
-      <c r="B27" s="50"/>
-      <c r="C27" s="50"/>
-      <c r="D27" s="50"/>
-      <c r="E27" s="50"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="50"/>
-      <c r="I27" s="51"/>
-      <c r="J27" s="51"/>
+      <c r="A27" s="50"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="52"/>
+      <c r="J27" s="52"/>
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:10">
-      <c r="B28" s="52"/>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
-      <c r="E28" s="52"/>
-      <c r="F28" s="52"/>
-      <c r="G28" s="53"/>
-      <c r="H28" s="53"/>
-      <c r="I28" s="54"/>
-      <c r="J28" s="54"/>
+      <c r="B28" s="53"/>
+      <c r="C28" s="53"/>
+      <c r="D28" s="53"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="53"/>
+      <c r="G28" s="54"/>
+      <c r="H28" s="54"/>
+      <c r="I28" s="55"/>
+      <c r="J28" s="55"/>
     </row>
     <row r="29" spans="1:10">
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="55"/>
-      <c r="H29" s="55"/>
-      <c r="I29" s="56"/>
-      <c r="J29" s="56"/>
+      <c r="C29" s="56"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="57"/>
     </row>
     <row r="30" spans="1:10">
-      <c r="B30" s="53"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="53"/>
-      <c r="E30" s="53"/>
-      <c r="F30" s="53"/>
-      <c r="G30" s="53"/>
-      <c r="H30" s="53"/>
-      <c r="I30" s="54"/>
-      <c r="J30" s="54"/>
+      <c r="B30" s="54"/>
+      <c r="C30" s="54"/>
+      <c r="D30" s="54"/>
+      <c r="E30" s="54"/>
+      <c r="F30" s="54"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="54"/>
+      <c r="I30" s="55"/>
+      <c r="J30" s="55"/>
     </row>
     <row r="31" spans="1:10">
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="53"/>
-      <c r="G31" s="53"/>
-      <c r="H31" s="53"/>
-      <c r="I31" s="54"/>
-      <c r="J31" s="54"/>
+      <c r="B31" s="54"/>
+      <c r="C31" s="54"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="54"/>
+      <c r="F31" s="54"/>
+      <c r="G31" s="54"/>
+      <c r="H31" s="54"/>
+      <c r="I31" s="55"/>
+      <c r="J31" s="55"/>
     </row>
     <row r="32" spans="1:10">
-      <c r="B32" s="53"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="53"/>
-      <c r="F32" s="53"/>
-      <c r="G32" s="53"/>
-      <c r="H32" s="53"/>
-      <c r="I32" s="54"/>
-      <c r="J32" s="54"/>
+      <c r="B32" s="54"/>
+      <c r="C32" s="54"/>
+      <c r="D32" s="54"/>
+      <c r="E32" s="54"/>
+      <c r="F32" s="54"/>
+      <c r="G32" s="54"/>
+      <c r="H32" s="54"/>
+      <c r="I32" s="55"/>
+      <c r="J32" s="55"/>
     </row>
     <row r="33" spans="2:10">
-      <c r="B33" s="53"/>
-      <c r="C33" s="53"/>
-      <c r="D33" s="53"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="53"/>
-      <c r="G33" s="53"/>
-      <c r="H33" s="53"/>
-      <c r="I33" s="54"/>
-      <c r="J33" s="54"/>
+      <c r="B33" s="54"/>
+      <c r="C33" s="54"/>
+      <c r="D33" s="54"/>
+      <c r="E33" s="54"/>
+      <c r="F33" s="54"/>
+      <c r="G33" s="54"/>
+      <c r="H33" s="54"/>
+      <c r="I33" s="55"/>
+      <c r="J33" s="55"/>
     </row>
     <row r="54" spans="3:3">
-      <c r="C54" s="57"/>
+      <c r="C54" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="47">

</xml_diff>

<commit_message>
chore: adopt latest fixed order template
</commit_message>
<xml_diff>
--- a/src/assets/order-templates/ROMIKU_订单_模板.xlsx
+++ b/src/assets/order-templates/ROMIKU_订单_模板.xlsx
@@ -10,7 +10,7 @@
     <sheet name="ROMIKU PI" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROMIKU PI'!$A$1:$J$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROMIKU PI'!$A$1:$J$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,9 +30,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="49">
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="36"/>
+        <rFont val="Songti SC Regular"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">                          </t>
     </r>
     <r>
@@ -94,6 +100,10 @@
   </si>
   <si>
     <t>info@romiku.com</t>
+  </si>
+  <si>
+    <t>订单要求
+REQUIREMENTS</t>
   </si>
   <si>
     <t>NO.
@@ -234,7 +244,7 @@
     <numFmt numFmtId="176" formatCode="\$#,##0.00;\-\$#,##0.00"/>
     <numFmt numFmtId="177" formatCode="&quot;USD&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -261,6 +271,24 @@
       <b/>
       <sz val="18"/>
       <name val="Songti SC Regular"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="28"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="36"/>
+      <name val="宋体"/>
       <charset val="134"/>
     </font>
     <font>
@@ -937,31 +965,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -970,120 +986,132 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyFont="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
@@ -1123,82 +1151,91 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="5" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="7" fontId="6" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="7" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="7" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="7" fontId="6" fillId="0" borderId="8" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="9" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="7" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="9" fillId="0" borderId="7" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="9" fillId="0" borderId="8" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="10" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="10" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="10" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="9" fillId="0" borderId="10" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="7" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="7" fontId="10" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="11" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="11" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="5" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1210,16 +1247,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1228,29 +1265,29 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="49" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="12" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="15" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="49" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="16" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="49" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1725,7 +1762,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="2" max="2" width="29.7788461538462" customWidth="1"/>
@@ -1814,7 +1851,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="9"/>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="62" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="11"/>
@@ -1863,441 +1900,455 @@
       <c r="I7" s="11"/>
       <c r="J7" s="12"/>
     </row>
-    <row r="8" ht="60" customHeight="1" spans="1:10">
+    <row r="8" ht="168" customHeight="1" spans="1:10">
       <c r="A8" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="16"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+    </row>
+    <row r="9" ht="60" customHeight="1" spans="1:10">
+      <c r="A9" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="B9" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="C9" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="D9" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="E9" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="16" t="s">
+      <c r="F9" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="16" t="s">
+      <c r="G9" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="17" t="s">
+      <c r="H9" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="17" t="s">
+      <c r="I9" s="20" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" ht="100" customHeight="1" spans="1:10">
-      <c r="A9" s="18">
+      <c r="J9" s="20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" ht="100" customHeight="1" spans="1:10">
+      <c r="A10" s="21">
         <v>1</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="21"/>
-    </row>
-    <row r="10" ht="100" customHeight="1" spans="1:10">
-      <c r="A10" s="18">
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="24"/>
+    </row>
+    <row r="11" ht="100" customHeight="1" spans="1:10">
+      <c r="A11" s="21">
         <v>2</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="18">
-        <f>G10*F10</f>
-        <v>0</v>
-      </c>
-      <c r="I10" s="23"/>
-      <c r="J10" s="24">
-        <f>H10*I10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" ht="100" customHeight="1" spans="1:10">
-      <c r="A11" s="18">
-        <v>3</v>
-      </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="18">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="21">
         <f>G11*F11</f>
         <v>0</v>
       </c>
-      <c r="I11" s="23"/>
-      <c r="J11" s="24">
+      <c r="I11" s="26"/>
+      <c r="J11" s="27">
         <f>H11*I11</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="100" customHeight="1" spans="1:10">
-      <c r="A12" s="25">
-        <v>4</v>
-      </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="25">
+      <c r="A12" s="21">
+        <v>3</v>
+      </c>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="21">
         <f>G12*F12</f>
         <v>0</v>
       </c>
-      <c r="I12" s="28"/>
-      <c r="J12" s="24">
+      <c r="I12" s="26"/>
+      <c r="J12" s="27">
         <f>H12*I12</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1" spans="1:10">
-      <c r="A13" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
+    <row r="13" ht="100" customHeight="1" spans="1:10">
+      <c r="A13" s="28">
+        <v>4</v>
+      </c>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
       <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="30">
-        <f>SUM(F9:F12)</f>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="28">
+        <f>G13*F13</f>
         <v>0</v>
       </c>
-      <c r="G13" s="31" t="s">
+      <c r="I13" s="31"/>
+      <c r="J13" s="27">
+        <f>H13*I13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1" spans="1:10">
+      <c r="A14" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="H13" s="31"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="33">
-        <f>SUM(J9:J12)</f>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="33">
+        <f>SUM(F10:F13)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" ht="45" customHeight="1" spans="1:10">
-      <c r="A14" s="34" t="s">
+      <c r="G14" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
+      <c r="H14" s="34"/>
       <c r="I14" s="35"/>
-      <c r="J14" s="33">
+      <c r="J14" s="36">
+        <f>SUM(J10:J13)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1" spans="1:10">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="33">
-        <f>J13+J14</f>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="36">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:10">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="33">
-        <f>J15*30%</f>
+      <c r="B16" s="39"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="39"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="36">
+        <f>J14+J15</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1" spans="1:10">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="38"/>
-      <c r="J17" s="33">
-        <f>J15-J16</f>
+      <c r="B17" s="32"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="36">
+        <f>J16*30%</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" spans="1:10">
-      <c r="A18" s="39" t="s">
+    <row r="18" ht="45" customHeight="1" spans="1:10">
+      <c r="A18" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="40"/>
-      <c r="J18" s="40"/>
-    </row>
-    <row r="19" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
-      <c r="A19" s="41">
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="36">
+        <f>J16-J17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1" spans="1:10">
+      <c r="A19" s="42" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43"/>
+    </row>
+    <row r="20" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
+      <c r="A20" s="44">
         <v>1</v>
       </c>
-      <c r="B19" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="43"/>
-      <c r="D19" s="44" t="s">
+      <c r="B20" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="46"/>
-      <c r="J19" s="47"/>
-    </row>
-    <row r="20" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
-      <c r="A20" s="41">
+      <c r="C20" s="46"/>
+      <c r="D20" s="47" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="48"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="50"/>
+    </row>
+    <row r="21" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
+      <c r="A21" s="44">
         <v>2</v>
       </c>
-      <c r="B20" s="48" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="49"/>
-      <c r="D20" s="44" t="s">
+      <c r="B21" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="E20" s="45"/>
-      <c r="F20" s="45"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="46"/>
-      <c r="J20" s="47"/>
-    </row>
-    <row r="21" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
-      <c r="A21" s="41">
+      <c r="C21" s="52"/>
+      <c r="D21" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
+      <c r="H21" s="48"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="50"/>
+    </row>
+    <row r="22" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
+      <c r="A22" s="44">
         <v>3</v>
       </c>
-      <c r="B21" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="49"/>
-      <c r="D21" s="44" t="s">
+      <c r="B22" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="47"/>
-    </row>
-    <row r="22" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
-      <c r="A22" s="41">
+      <c r="C22" s="52"/>
+      <c r="D22" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="50"/>
+    </row>
+    <row r="23" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
+      <c r="A23" s="44">
         <v>4</v>
       </c>
-      <c r="B22" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="49"/>
-      <c r="D22" s="44" t="s">
+      <c r="B23" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="45"/>
-      <c r="J22" s="47"/>
-    </row>
-    <row r="23" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
-      <c r="A23" s="41">
+      <c r="C23" s="52"/>
+      <c r="D23" s="47" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="48"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="50"/>
+    </row>
+    <row r="24" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
+      <c r="A24" s="44">
         <v>5</v>
       </c>
-      <c r="B23" s="48" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="49"/>
-      <c r="D23" s="44" t="s">
+      <c r="B24" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="47"/>
-    </row>
-    <row r="24" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
-      <c r="A24" s="41">
+      <c r="C24" s="52"/>
+      <c r="D24" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="48"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="50"/>
+    </row>
+    <row r="25" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
+      <c r="A25" s="44">
         <v>6</v>
       </c>
-      <c r="B24" s="48" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" s="49"/>
-      <c r="D24" s="44" t="s">
+      <c r="B25" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="45"/>
-      <c r="J24" s="47"/>
-    </row>
-    <row r="25" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
-      <c r="A25" s="41">
+      <c r="C25" s="52"/>
+      <c r="D25" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="48"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="50"/>
+    </row>
+    <row r="26" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
+      <c r="A26" s="44">
         <v>7</v>
       </c>
-      <c r="B25" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="43"/>
-      <c r="D25" s="44" t="s">
+      <c r="B26" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="45"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="47"/>
-    </row>
-    <row r="26" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
-      <c r="A26" s="41">
+      <c r="C26" s="46"/>
+      <c r="D26" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26" s="48"/>
+      <c r="F26" s="48"/>
+      <c r="G26" s="48"/>
+      <c r="H26" s="48"/>
+      <c r="I26" s="49"/>
+      <c r="J26" s="50"/>
+    </row>
+    <row r="27" s="1" customFormat="1" ht="75" customHeight="1" spans="1:10">
+      <c r="A27" s="44">
         <v>8</v>
       </c>
-      <c r="B26" s="42" t="s">
-        <v>46</v>
-      </c>
-      <c r="C26" s="43"/>
-      <c r="D26" s="44" t="s">
+      <c r="B27" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="45"/>
-      <c r="I26" s="46"/>
-      <c r="J26" s="47"/>
-    </row>
-    <row r="27" s="1" customFormat="1" ht="24" customHeight="1" spans="1:10">
-      <c r="A27" s="50"/>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="51"/>
-      <c r="H27" s="51"/>
-      <c r="I27" s="52"/>
-      <c r="J27" s="52"/>
-    </row>
-    <row r="28" ht="40" customHeight="1" spans="1:10">
-      <c r="B28" s="53"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="53"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="53"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="47" t="s">
+        <v>48</v>
+      </c>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="G27" s="48"/>
+      <c r="H27" s="48"/>
+      <c r="I27" s="49"/>
+      <c r="J27" s="50"/>
+    </row>
+    <row r="28" s="1" customFormat="1" ht="24" customHeight="1" spans="1:10">
+      <c r="A28" s="53"/>
+      <c r="B28" s="54"/>
+      <c r="C28" s="54"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="54"/>
+      <c r="F28" s="54"/>
       <c r="G28" s="54"/>
       <c r="H28" s="54"/>
       <c r="I28" s="55"/>
       <c r="J28" s="55"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" ht="40" customHeight="1" spans="1:10">
+      <c r="B29" s="56"/>
       <c r="C29" s="56"/>
       <c r="D29" s="56"/>
       <c r="E29" s="56"/>
       <c r="F29" s="56"/>
-      <c r="G29" s="56"/>
-      <c r="H29" s="56"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="57"/>
+      <c r="G29" s="57"/>
+      <c r="H29" s="57"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="58"/>
     </row>
     <row r="30" spans="1:10">
-      <c r="B30" s="54"/>
-      <c r="C30" s="54"/>
-      <c r="D30" s="54"/>
-      <c r="E30" s="54"/>
-      <c r="F30" s="54"/>
-      <c r="G30" s="54"/>
-      <c r="H30" s="54"/>
-      <c r="I30" s="55"/>
-      <c r="J30" s="55"/>
+      <c r="C30" s="59"/>
+      <c r="D30" s="59"/>
+      <c r="E30" s="59"/>
+      <c r="F30" s="59"/>
+      <c r="G30" s="59"/>
+      <c r="H30" s="59"/>
+      <c r="I30" s="60"/>
+      <c r="J30" s="60"/>
     </row>
     <row r="31" spans="1:10">
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="54"/>
-      <c r="E31" s="54"/>
-      <c r="F31" s="54"/>
-      <c r="G31" s="54"/>
-      <c r="H31" s="54"/>
-      <c r="I31" s="55"/>
-      <c r="J31" s="55"/>
+      <c r="B31" s="57"/>
+      <c r="C31" s="57"/>
+      <c r="D31" s="57"/>
+      <c r="E31" s="57"/>
+      <c r="F31" s="57"/>
+      <c r="G31" s="57"/>
+      <c r="H31" s="57"/>
+      <c r="I31" s="58"/>
+      <c r="J31" s="58"/>
     </row>
     <row r="32" spans="1:10">
-      <c r="B32" s="54"/>
-      <c r="C32" s="54"/>
-      <c r="D32" s="54"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="54"/>
-      <c r="G32" s="54"/>
-      <c r="H32" s="54"/>
-      <c r="I32" s="55"/>
-      <c r="J32" s="55"/>
+      <c r="B32" s="57"/>
+      <c r="C32" s="57"/>
+      <c r="D32" s="57"/>
+      <c r="E32" s="57"/>
+      <c r="F32" s="57"/>
+      <c r="G32" s="57"/>
+      <c r="H32" s="57"/>
+      <c r="I32" s="58"/>
+      <c r="J32" s="58"/>
     </row>
     <row r="33" spans="2:10">
-      <c r="B33" s="54"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="54"/>
-      <c r="E33" s="54"/>
-      <c r="F33" s="54"/>
-      <c r="G33" s="54"/>
-      <c r="H33" s="54"/>
-      <c r="I33" s="55"/>
-      <c r="J33" s="55"/>
-    </row>
-    <row r="54" spans="3:3">
-      <c r="C54" s="58"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="57"/>
+      <c r="D33" s="57"/>
+      <c r="E33" s="57"/>
+      <c r="F33" s="57"/>
+      <c r="G33" s="57"/>
+      <c r="H33" s="57"/>
+      <c r="I33" s="58"/>
+      <c r="J33" s="58"/>
+    </row>
+    <row r="34" spans="2:10">
+      <c r="B34" s="57"/>
+      <c r="C34" s="57"/>
+      <c r="D34" s="57"/>
+      <c r="E34" s="57"/>
+      <c r="F34" s="57"/>
+      <c r="G34" s="57"/>
+      <c r="H34" s="57"/>
+      <c r="I34" s="58"/>
+      <c r="J34" s="58"/>
+    </row>
+    <row r="55" spans="3:3">
+      <c r="C55" s="61"/>
     </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="49">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="F2:J2"/>
@@ -2321,15 +2372,15 @@
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="H7:J7"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="G14:I14"/>
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A16:I16"/>
     <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A18:J18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:J19"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A19:J19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="D20:J20"/>
     <mergeCell ref="B21:C21"/>
@@ -2344,7 +2395,9 @@
     <mergeCell ref="D25:J25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="D26:J26"/>
-    <mergeCell ref="B27:J27"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:J27"/>
+    <mergeCell ref="B28:J28"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.12" footer="0.12"/>

</xml_diff>